<commit_message>
2024 Temmuz Günce maaş Katsayıları eklendi.
</commit_message>
<xml_diff>
--- a/maas_verileri.xlsx
+++ b/maas_verileri.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId3"/>
@@ -911,7 +911,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="10.46"/>
@@ -1478,6 +1478,20 @@
       </c>
       <c r="D40" s="2" t="n">
         <v>11.909083</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="n">
+        <v>45474</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>0.907796</v>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>0.287892</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>14.208727</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bazı hatalar giderildi. Eğitim uzmanı unvanı, KBS ile uyumlu hale getirildi ve ayn ödemeleri eklendi.
</commit_message>
<xml_diff>
--- a/maas_verileri.xlsx
+++ b/maas_verileri.xlsx
@@ -8,10 +8,10 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="maas_kat_sayilari" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="yan_odeme_puanlari" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="ozel_hizmet_tazminati" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="maas_kat_sayilari" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="yan_odeme_puanlari" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="ozel_hizmet_tazminati" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="59">
   <si>
     <t xml:space="preserve">yil</t>
   </si>
@@ -118,6 +118,9 @@
     <t xml:space="preserve">Din Hz.Uzm</t>
   </si>
   <si>
+    <t xml:space="preserve">Eğt.Uzmanı</t>
+  </si>
+  <si>
     <t xml:space="preserve">Memur</t>
   </si>
   <si>
@@ -187,9 +190,6 @@
     <t xml:space="preserve">ogrenim</t>
   </si>
   <si>
-    <t xml:space="preserve">Eğitim Uzmanı</t>
-  </si>
-  <si>
     <t xml:space="preserve">Yüksek Okul</t>
   </si>
   <si>
@@ -211,7 +211,7 @@
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -238,6 +238,13 @@
       <sz val="12"/>
       <name val="Times New Roman Tur"/>
       <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -283,7 +290,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -328,6 +335,10 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -338,112 +349,6 @@
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
 </styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="LibreOffice">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="000000"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="ffffff"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="18a303"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="0369a3"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="a33e03"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8e03a3"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="c99c00"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="c9211e"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000ee"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="551a8b"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1510,7 +1415,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="35.58"/>
@@ -2066,100 +1971,127 @@
         <v>1</v>
       </c>
       <c r="C38" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B40" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C40" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C41" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B42" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C42" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B43" s="1" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C43" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B44" s="1" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C44" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
+      </c>
+      <c r="E44" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B45" s="1" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C45" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
+      </c>
+      <c r="E45" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B46" s="1" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C46" s="1" t="n">
-        <v>500</v>
+        <v>600</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>1</v>
@@ -2170,7 +2102,7 @@
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>1</v>
@@ -2181,7 +2113,7 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>1</v>
@@ -2192,7 +2124,7 @@
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B50" s="1" t="n">
         <v>1</v>
@@ -2200,13 +2132,10 @@
       <c r="C50" s="1" t="n">
         <v>500</v>
       </c>
-      <c r="D50" s="1" t="n">
-        <v>175</v>
-      </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="B51" s="1" t="n">
         <v>1</v>
@@ -2217,7 +2146,7 @@
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B52" s="1" t="n">
         <v>1</v>
@@ -2228,7 +2157,7 @@
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B53" s="1" t="n">
         <v>1</v>
@@ -2239,7 +2168,7 @@
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B54" s="1" t="n">
         <v>1</v>
@@ -2250,7 +2179,7 @@
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B55" s="1" t="n">
         <v>1</v>
@@ -2261,64 +2190,166 @@
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B56" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="1" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B57" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="1" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" s="1" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B59" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" s="1" t="n">
+        <v>500</v>
+      </c>
+      <c r="D59" s="1" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B60" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" s="1" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B61" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" s="1" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B62" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B63" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" s="1" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B56" s="6" t="n">
+      <c r="B64" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C56" s="6" t="n">
+      <c r="C64" s="1" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-    </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-    </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-    </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-    </row>
-    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
-    </row>
-    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B71" s="2"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-      <c r="E71" s="2"/>
-    </row>
-    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B72" s="2"/>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-      <c r="E72" s="2"/>
-    </row>
-    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B73" s="2"/>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
-    </row>
-    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B74" s="2"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-    </row>
-    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B75" s="2"/>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B65" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="2"/>
+      <c r="C68" s="2"/>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="2"/>
+      <c r="C69" s="2"/>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="2"/>
+      <c r="C70" s="2"/>
+    </row>
+    <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="2"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="2"/>
+      <c r="E80" s="2"/>
+    </row>
+    <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B81" s="2"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
+      <c r="E81" s="2"/>
+    </row>
+    <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B82" s="2"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2"/>
+      <c r="E82" s="2"/>
+    </row>
+    <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B83" s="2"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
+      <c r="E83" s="2"/>
+    </row>
+    <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B84" s="2"/>
+      <c r="C84" s="2"/>
+      <c r="D84" s="2"/>
+      <c r="E84" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2357,16 +2388,16 @@
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2972,9 +3003,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="s">
-        <v>54</v>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>1</v>
@@ -2986,9 +3017,9 @@
         <v>115</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="s">
-        <v>54</v>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>2</v>
@@ -3000,9 +3031,9 @@
         <v>115</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="s">
-        <v>54</v>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>3</v>
@@ -3014,9 +3045,9 @@
         <v>110</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="s">
-        <v>54</v>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="B48" s="1" t="n">
         <v>4</v>
@@ -3028,9 +3059,9 @@
         <v>110</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="s">
-        <v>54</v>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="B49" s="1" t="n">
         <v>5</v>
@@ -4838,7 +4869,7 @@
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B158" s="1" t="n">
         <v>1</v>
@@ -4858,7 +4889,7 @@
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B159" s="1" t="n">
         <v>2</v>
@@ -4878,7 +4909,7 @@
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B160" s="1" t="n">
         <v>3</v>
@@ -4898,7 +4929,7 @@
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B161" s="1" t="n">
         <v>4</v>
@@ -4918,7 +4949,7 @@
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B162" s="1" t="n">
         <v>1</v>
@@ -4938,7 +4969,7 @@
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B163" s="1" t="n">
         <v>2</v>
@@ -4958,7 +4989,7 @@
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B164" s="1" t="n">
         <v>3</v>
@@ -4978,7 +5009,7 @@
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B165" s="1" t="n">
         <v>4</v>
@@ -4998,7 +5029,7 @@
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B166" s="1" t="n">
         <v>5</v>
@@ -5018,7 +5049,7 @@
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B167" s="1" t="n">
         <v>6</v>
@@ -5038,7 +5069,7 @@
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B168" s="1" t="n">
         <v>1</v>
@@ -5055,7 +5086,7 @@
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B169" s="1" t="n">
         <v>2</v>
@@ -5072,7 +5103,7 @@
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B170" s="1" t="n">
         <v>3</v>
@@ -5089,7 +5120,7 @@
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B171" s="1" t="n">
         <v>4</v>
@@ -5106,7 +5137,7 @@
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B172" s="1" t="n">
         <v>5</v>
@@ -5123,7 +5154,7 @@
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B173" s="1" t="n">
         <v>6</v>
@@ -5140,7 +5171,7 @@
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B174" s="1" t="n">
         <v>7</v>
@@ -5157,7 +5188,7 @@
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B175" s="1" t="n">
         <v>8</v>
@@ -5174,7 +5205,7 @@
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B176" s="1" t="n">
         <v>9</v>
@@ -5191,7 +5222,7 @@
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B177" s="1" t="n">
         <v>10</v>
@@ -5208,7 +5239,7 @@
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B178" s="1" t="n">
         <v>11</v>
@@ -5225,7 +5256,7 @@
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B179" s="1" t="n">
         <v>12</v>
@@ -5242,7 +5273,7 @@
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B180" s="1" t="n">
         <v>13</v>
@@ -5259,7 +5290,7 @@
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B181" s="1" t="n">
         <v>14</v>
@@ -5276,7 +5307,7 @@
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B182" s="1" t="n">
         <v>15</v>
@@ -5293,7 +5324,7 @@
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B183" s="1" t="n">
         <v>1</v>
@@ -5310,7 +5341,7 @@
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B184" s="1" t="n">
         <v>2</v>
@@ -5327,7 +5358,7 @@
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B185" s="1" t="n">
         <v>3</v>
@@ -5344,7 +5375,7 @@
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B186" s="1" t="n">
         <v>4</v>
@@ -5361,7 +5392,7 @@
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B187" s="1" t="n">
         <v>5</v>
@@ -5378,7 +5409,7 @@
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B188" s="1" t="n">
         <v>6</v>
@@ -5395,7 +5426,7 @@
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B189" s="1" t="n">
         <v>7</v>
@@ -5412,7 +5443,7 @@
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B190" s="1" t="n">
         <v>8</v>
@@ -5429,7 +5460,7 @@
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B191" s="1" t="n">
         <v>9</v>
@@ -5446,7 +5477,7 @@
     </row>
     <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B192" s="1" t="n">
         <v>10</v>
@@ -5463,7 +5494,7 @@
     </row>
     <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B193" s="1" t="n">
         <v>11</v>
@@ -5480,7 +5511,7 @@
     </row>
     <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B194" s="1" t="n">
         <v>12</v>
@@ -5497,7 +5528,7 @@
     </row>
     <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B195" s="1" t="n">
         <v>13</v>
@@ -5514,7 +5545,7 @@
     </row>
     <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B196" s="1" t="n">
         <v>14</v>
@@ -5531,7 +5562,7 @@
     </row>
     <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B197" s="1" t="n">
         <v>15</v>
@@ -5548,7 +5579,7 @@
     </row>
     <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B198" s="1" t="n">
         <v>1</v>
@@ -5565,7 +5596,7 @@
     </row>
     <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B199" s="1" t="n">
         <v>2</v>
@@ -5582,7 +5613,7 @@
     </row>
     <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B200" s="1" t="n">
         <v>3</v>
@@ -5599,7 +5630,7 @@
     </row>
     <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B201" s="1" t="n">
         <v>4</v>
@@ -5616,7 +5647,7 @@
     </row>
     <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B202" s="1" t="n">
         <v>5</v>
@@ -5633,7 +5664,7 @@
     </row>
     <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B203" s="1" t="n">
         <v>6</v>
@@ -5650,7 +5681,7 @@
     </row>
     <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B204" s="1" t="n">
         <v>7</v>
@@ -5667,7 +5698,7 @@
     </row>
     <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B205" s="1" t="n">
         <v>8</v>
@@ -5684,7 +5715,7 @@
     </row>
     <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B206" s="1" t="n">
         <v>9</v>
@@ -5701,7 +5732,7 @@
     </row>
     <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B207" s="1" t="n">
         <v>10</v>
@@ -5718,7 +5749,7 @@
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B208" s="1" t="n">
         <v>11</v>
@@ -5735,7 +5766,7 @@
     </row>
     <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B209" s="1" t="n">
         <v>12</v>
@@ -5752,7 +5783,7 @@
     </row>
     <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B210" s="1" t="n">
         <v>13</v>
@@ -5769,7 +5800,7 @@
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B211" s="1" t="n">
         <v>14</v>
@@ -5786,7 +5817,7 @@
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B212" s="1" t="n">
         <v>15</v>
@@ -5803,7 +5834,7 @@
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B213" s="1" t="n">
         <v>1</v>
@@ -5823,7 +5854,7 @@
     </row>
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B214" s="1" t="n">
         <v>2</v>
@@ -5843,7 +5874,7 @@
     </row>
     <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B215" s="1" t="n">
         <v>3</v>
@@ -5863,7 +5894,7 @@
     </row>
     <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B216" s="1" t="n">
         <v>4</v>
@@ -5883,7 +5914,7 @@
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B217" s="1" t="n">
         <v>1</v>
@@ -5900,7 +5931,7 @@
     </row>
     <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B218" s="1" t="n">
         <v>2</v>
@@ -5917,7 +5948,7 @@
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B219" s="1" t="n">
         <v>3</v>
@@ -5934,7 +5965,7 @@
     </row>
     <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B220" s="1" t="n">
         <v>4</v>
@@ -5951,7 +5982,7 @@
     </row>
     <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B221" s="1" t="n">
         <v>5</v>
@@ -5968,7 +5999,7 @@
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B222" s="1" t="n">
         <v>6</v>
@@ -5985,7 +6016,7 @@
     </row>
     <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B223" s="1" t="n">
         <v>7</v>
@@ -6002,7 +6033,7 @@
     </row>
     <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B224" s="1" t="n">
         <v>8</v>
@@ -6019,7 +6050,7 @@
     </row>
     <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B225" s="1" t="n">
         <v>9</v>
@@ -6036,7 +6067,7 @@
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B226" s="1" t="n">
         <v>10</v>
@@ -6053,7 +6084,7 @@
     </row>
     <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B227" s="1" t="n">
         <v>11</v>
@@ -6070,7 +6101,7 @@
     </row>
     <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B228" s="1" t="n">
         <v>12</v>
@@ -6087,7 +6118,7 @@
     </row>
     <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B229" s="1" t="n">
         <v>13</v>
@@ -6104,7 +6135,7 @@
     </row>
     <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B230" s="1" t="n">
         <v>14</v>
@@ -6121,7 +6152,7 @@
     </row>
     <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B231" s="1" t="n">
         <v>15</v>
@@ -6138,7 +6169,7 @@
     </row>
     <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B232" s="1" t="n">
         <v>1</v>
@@ -6155,7 +6186,7 @@
     </row>
     <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B233" s="1" t="n">
         <v>2</v>
@@ -6172,7 +6203,7 @@
     </row>
     <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B234" s="1" t="n">
         <v>3</v>
@@ -6189,7 +6220,7 @@
     </row>
     <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B235" s="1" t="n">
         <v>4</v>
@@ -6206,7 +6237,7 @@
     </row>
     <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B236" s="1" t="n">
         <v>5</v>
@@ -6223,7 +6254,7 @@
     </row>
     <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B237" s="1" t="n">
         <v>6</v>
@@ -6240,7 +6271,7 @@
     </row>
     <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B238" s="1" t="n">
         <v>7</v>
@@ -6257,7 +6288,7 @@
     </row>
     <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B239" s="1" t="n">
         <v>8</v>
@@ -6274,7 +6305,7 @@
     </row>
     <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B240" s="1" t="n">
         <v>9</v>
@@ -6291,7 +6322,7 @@
     </row>
     <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B241" s="1" t="n">
         <v>10</v>
@@ -6308,7 +6339,7 @@
     </row>
     <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B242" s="1" t="n">
         <v>11</v>
@@ -6325,7 +6356,7 @@
     </row>
     <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B243" s="1" t="n">
         <v>12</v>
@@ -6342,7 +6373,7 @@
     </row>
     <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B244" s="1" t="n">
         <v>13</v>
@@ -6359,7 +6390,7 @@
     </row>
     <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B245" s="1" t="n">
         <v>14</v>
@@ -6376,7 +6407,7 @@
     </row>
     <row r="246" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B246" s="1" t="n">
         <v>15</v>
@@ -6393,7 +6424,7 @@
     </row>
     <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B247" s="1" t="n">
         <v>1</v>
@@ -6410,7 +6441,7 @@
     </row>
     <row r="248" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B248" s="1" t="n">
         <v>2</v>
@@ -6427,7 +6458,7 @@
     </row>
     <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B249" s="1" t="n">
         <v>3</v>
@@ -6444,7 +6475,7 @@
     </row>
     <row r="250" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B250" s="1" t="n">
         <v>4</v>
@@ -6461,7 +6492,7 @@
     </row>
     <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B251" s="1" t="n">
         <v>5</v>
@@ -6478,7 +6509,7 @@
     </row>
     <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B252" s="1" t="n">
         <v>6</v>
@@ -6495,7 +6526,7 @@
     </row>
     <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B253" s="1" t="n">
         <v>7</v>
@@ -6512,7 +6543,7 @@
     </row>
     <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B254" s="1" t="n">
         <v>8</v>
@@ -6529,7 +6560,7 @@
     </row>
     <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B255" s="1" t="n">
         <v>9</v>
@@ -6546,7 +6577,7 @@
     </row>
     <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B256" s="1" t="n">
         <v>10</v>
@@ -6563,7 +6594,7 @@
     </row>
     <row r="257" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B257" s="1" t="n">
         <v>11</v>
@@ -6580,7 +6611,7 @@
     </row>
     <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B258" s="1" t="n">
         <v>12</v>
@@ -6597,7 +6628,7 @@
     </row>
     <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B259" s="1" t="n">
         <v>13</v>
@@ -6614,7 +6645,7 @@
     </row>
     <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B260" s="1" t="n">
         <v>14</v>
@@ -6631,7 +6662,7 @@
     </row>
     <row r="261" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B261" s="1" t="n">
         <v>15</v>
@@ -6648,7 +6679,7 @@
     </row>
     <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B262" s="1" t="n">
         <v>1</v>
@@ -6668,7 +6699,7 @@
     </row>
     <row r="263" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B263" s="1" t="n">
         <v>2</v>
@@ -6688,7 +6719,7 @@
     </row>
     <row r="264" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B264" s="1" t="n">
         <v>3</v>
@@ -6708,7 +6739,7 @@
     </row>
     <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B265" s="1" t="n">
         <v>4</v>
@@ -6728,7 +6759,7 @@
     </row>
     <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B266" s="1" t="n">
         <v>1</v>
@@ -6748,7 +6779,7 @@
     </row>
     <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B267" s="1" t="n">
         <v>2</v>
@@ -6768,7 +6799,7 @@
     </row>
     <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B268" s="1" t="n">
         <v>3</v>
@@ -6788,7 +6819,7 @@
     </row>
     <row r="269" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B269" s="1" t="n">
         <v>4</v>
@@ -6808,7 +6839,7 @@
     </row>
     <row r="270" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A270" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B270" s="1" t="n">
         <v>5</v>
@@ -6828,7 +6859,7 @@
     </row>
     <row r="271" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B271" s="1" t="n">
         <v>6</v>
@@ -6848,7 +6879,7 @@
     </row>
     <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B272" s="1" t="n">
         <v>7</v>
@@ -6868,7 +6899,7 @@
     </row>
     <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B273" s="1" t="n">
         <v>8</v>
@@ -6888,7 +6919,7 @@
     </row>
     <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B274" s="1" t="n">
         <v>1</v>
@@ -6905,7 +6936,7 @@
     </row>
     <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B275" s="1" t="n">
         <v>2</v>
@@ -6922,7 +6953,7 @@
     </row>
     <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B276" s="1" t="n">
         <v>3</v>
@@ -6939,7 +6970,7 @@
     </row>
     <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B277" s="1" t="n">
         <v>4</v>
@@ -6956,7 +6987,7 @@
     </row>
     <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B278" s="1" t="n">
         <v>5</v>
@@ -6973,7 +7004,7 @@
     </row>
     <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B279" s="1" t="n">
         <v>6</v>
@@ -6990,7 +7021,7 @@
     </row>
     <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B280" s="1" t="n">
         <v>7</v>
@@ -7007,7 +7038,7 @@
     </row>
     <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B281" s="1" t="n">
         <v>8</v>
@@ -7024,7 +7055,7 @@
     </row>
     <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B282" s="1" t="n">
         <v>9</v>
@@ -7041,7 +7072,7 @@
     </row>
     <row r="283" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B283" s="1" t="n">
         <v>10</v>
@@ -7058,7 +7089,7 @@
     </row>
     <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B284" s="1" t="n">
         <v>11</v>
@@ -7075,7 +7106,7 @@
     </row>
     <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B285" s="1" t="n">
         <v>12</v>
@@ -7092,7 +7123,7 @@
     </row>
     <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B286" s="1" t="n">
         <v>13</v>
@@ -7109,7 +7140,7 @@
     </row>
     <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B287" s="1" t="n">
         <v>14</v>
@@ -7126,7 +7157,7 @@
     </row>
     <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B288" s="1" t="n">
         <v>15</v>
@@ -7143,7 +7174,7 @@
     </row>
     <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B289" s="1" t="n">
         <v>1</v>
@@ -7160,7 +7191,7 @@
     </row>
     <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B290" s="1" t="n">
         <v>2</v>
@@ -7177,7 +7208,7 @@
     </row>
     <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B291" s="1" t="n">
         <v>3</v>
@@ -7194,7 +7225,7 @@
     </row>
     <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B292" s="1" t="n">
         <v>4</v>
@@ -7211,7 +7242,7 @@
     </row>
     <row r="293" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B293" s="1" t="n">
         <v>5</v>
@@ -7228,7 +7259,7 @@
     </row>
     <row r="294" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A294" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B294" s="1" t="n">
         <v>6</v>
@@ -7245,7 +7276,7 @@
     </row>
     <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A295" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B295" s="1" t="n">
         <v>7</v>
@@ -7262,7 +7293,7 @@
     </row>
     <row r="296" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B296" s="1" t="n">
         <v>8</v>
@@ -7279,7 +7310,7 @@
     </row>
     <row r="297" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A297" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B297" s="1" t="n">
         <v>9</v>
@@ -7296,7 +7327,7 @@
     </row>
     <row r="298" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B298" s="1" t="n">
         <v>10</v>
@@ -7313,7 +7344,7 @@
     </row>
     <row r="299" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B299" s="1" t="n">
         <v>11</v>
@@ -7330,7 +7361,7 @@
     </row>
     <row r="300" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A300" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B300" s="1" t="n">
         <v>12</v>
@@ -7347,7 +7378,7 @@
     </row>
     <row r="301" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A301" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B301" s="1" t="n">
         <v>13</v>
@@ -7364,7 +7395,7 @@
     </row>
     <row r="302" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A302" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B302" s="1" t="n">
         <v>14</v>
@@ -7381,7 +7412,7 @@
     </row>
     <row r="303" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A303" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B303" s="1" t="n">
         <v>15</v>
@@ -7398,7 +7429,7 @@
     </row>
     <row r="304" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A304" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B304" s="1" t="n">
         <v>1</v>
@@ -7415,7 +7446,7 @@
     </row>
     <row r="305" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B305" s="1" t="n">
         <v>2</v>
@@ -7432,7 +7463,7 @@
     </row>
     <row r="306" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A306" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B306" s="1" t="n">
         <v>3</v>
@@ -7449,7 +7480,7 @@
     </row>
     <row r="307" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A307" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B307" s="1" t="n">
         <v>4</v>
@@ -7466,7 +7497,7 @@
     </row>
     <row r="308" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A308" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B308" s="1" t="n">
         <v>5</v>
@@ -7483,7 +7514,7 @@
     </row>
     <row r="309" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A309" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B309" s="1" t="n">
         <v>6</v>
@@ -7500,7 +7531,7 @@
     </row>
     <row r="310" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A310" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B310" s="1" t="n">
         <v>7</v>
@@ -7517,7 +7548,7 @@
     </row>
     <row r="311" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A311" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B311" s="1" t="n">
         <v>8</v>
@@ -7534,7 +7565,7 @@
     </row>
     <row r="312" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A312" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B312" s="1" t="n">
         <v>9</v>
@@ -7551,7 +7582,7 @@
     </row>
     <row r="313" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B313" s="1" t="n">
         <v>10</v>
@@ -7568,7 +7599,7 @@
     </row>
     <row r="314" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A314" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B314" s="1" t="n">
         <v>11</v>
@@ -7585,7 +7616,7 @@
     </row>
     <row r="315" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A315" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B315" s="1" t="n">
         <v>12</v>
@@ -7602,7 +7633,7 @@
     </row>
     <row r="316" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A316" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B316" s="1" t="n">
         <v>13</v>
@@ -7619,7 +7650,7 @@
     </row>
     <row r="317" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A317" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B317" s="1" t="n">
         <v>14</v>
@@ -7636,7 +7667,7 @@
     </row>
     <row r="318" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A318" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B318" s="1" t="n">
         <v>15</v>
@@ -7653,7 +7684,7 @@
     </row>
     <row r="319" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A319" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B319" s="1" t="n">
         <v>1</v>
@@ -7667,7 +7698,7 @@
     </row>
     <row r="320" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A320" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B320" s="1" t="n">
         <v>2</v>
@@ -7681,7 +7712,7 @@
     </row>
     <row r="321" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B321" s="1" t="n">
         <v>3</v>
@@ -7695,7 +7726,7 @@
     </row>
     <row r="322" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A322" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B322" s="1" t="n">
         <v>4</v>
@@ -7709,7 +7740,7 @@
     </row>
     <row r="323" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A323" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B323" s="1" t="n">
         <v>5</v>
@@ -7723,7 +7754,7 @@
     </row>
     <row r="324" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A324" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B324" s="1" t="n">
         <v>6</v>
@@ -7737,7 +7768,7 @@
     </row>
     <row r="325" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A325" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B325" s="1" t="n">
         <v>7</v>
@@ -7751,7 +7782,7 @@
     </row>
     <row r="326" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B326" s="1" t="n">
         <v>8</v>
@@ -7765,7 +7796,7 @@
     </row>
     <row r="327" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A327" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B327" s="1" t="n">
         <v>9</v>
@@ -7779,7 +7810,7 @@
     </row>
     <row r="328" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A328" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B328" s="1" t="n">
         <v>10</v>
@@ -7793,7 +7824,7 @@
     </row>
     <row r="329" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A329" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B329" s="1" t="n">
         <v>11</v>
@@ -7807,7 +7838,7 @@
     </row>
     <row r="330" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A330" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B330" s="1" t="n">
         <v>12</v>
@@ -7821,7 +7852,7 @@
     </row>
     <row r="331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A331" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B331" s="1" t="n">
         <v>1</v>
@@ -7835,7 +7866,7 @@
     </row>
     <row r="332" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A332" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B332" s="1" t="n">
         <v>2</v>
@@ -7849,7 +7880,7 @@
     </row>
     <row r="333" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A333" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B333" s="1" t="n">
         <v>3</v>
@@ -7863,7 +7894,7 @@
     </row>
     <row r="334" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A334" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B334" s="1" t="n">
         <v>4</v>
@@ -7877,7 +7908,7 @@
     </row>
     <row r="335" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A335" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B335" s="1" t="n">
         <v>5</v>
@@ -7891,7 +7922,7 @@
     </row>
     <row r="336" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A336" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B336" s="1" t="n">
         <v>6</v>
@@ -7905,7 +7936,7 @@
     </row>
     <row r="337" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A337" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B337" s="1" t="n">
         <v>7</v>
@@ -7919,7 +7950,7 @@
     </row>
     <row r="338" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A338" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B338" s="1" t="n">
         <v>8</v>
@@ -7933,7 +7964,7 @@
     </row>
     <row r="339" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A339" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B339" s="1" t="n">
         <v>9</v>
@@ -7947,7 +7978,7 @@
     </row>
     <row r="340" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A340" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B340" s="1" t="n">
         <v>10</v>
@@ -7961,7 +7992,7 @@
     </row>
     <row r="341" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A341" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B341" s="1" t="n">
         <v>11</v>
@@ -7975,7 +8006,7 @@
     </row>
     <row r="342" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A342" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B342" s="1" t="n">
         <v>12</v>
@@ -7989,7 +8020,7 @@
     </row>
     <row r="343" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A343" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B343" s="1" t="n">
         <v>13</v>
@@ -8003,7 +8034,7 @@
     </row>
     <row r="344" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B344" s="1" t="n">
         <v>14</v>
@@ -8017,7 +8048,7 @@
     </row>
     <row r="345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B345" s="1" t="n">
         <v>15</v>
@@ -8143,7 +8174,7 @@
     </row>
     <row r="354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A354" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B354" s="1" t="n">
         <v>1</v>
@@ -8157,7 +8188,7 @@
     </row>
     <row r="355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A355" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B355" s="1" t="n">
         <v>2</v>
@@ -8171,7 +8202,7 @@
     </row>
     <row r="356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A356" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B356" s="1" t="n">
         <v>3</v>
@@ -8185,7 +8216,7 @@
     </row>
     <row r="357" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A357" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B357" s="1" t="n">
         <v>4</v>
@@ -8199,7 +8230,7 @@
     </row>
     <row r="358" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B358" s="1" t="n">
         <v>5</v>
@@ -8213,7 +8244,7 @@
     </row>
     <row r="359" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A359" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B359" s="1" t="n">
         <v>6</v>
@@ -8227,7 +8258,7 @@
     </row>
     <row r="360" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A360" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B360" s="1" t="n">
         <v>7</v>
@@ -8241,7 +8272,7 @@
     </row>
     <row r="361" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B361" s="1" t="n">
         <v>8</v>
@@ -8255,7 +8286,7 @@
     </row>
     <row r="362" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A362" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B362" s="1" t="n">
         <v>1</v>
@@ -8269,7 +8300,7 @@
     </row>
     <row r="363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A363" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B363" s="1" t="n">
         <v>2</v>
@@ -8283,7 +8314,7 @@
     </row>
     <row r="364" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A364" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B364" s="1" t="n">
         <v>3</v>
@@ -8297,7 +8328,7 @@
     </row>
     <row r="365" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B365" s="1" t="n">
         <v>4</v>
@@ -8311,7 +8342,7 @@
     </row>
     <row r="366" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A366" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B366" s="1" t="n">
         <v>5</v>
@@ -8325,7 +8356,7 @@
     </row>
     <row r="367" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B367" s="1" t="n">
         <v>6</v>
@@ -8339,7 +8370,7 @@
     </row>
     <row r="368" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A368" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B368" s="1" t="n">
         <v>7</v>
@@ -8353,7 +8384,7 @@
     </row>
     <row r="369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A369" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B369" s="1" t="n">
         <v>8</v>
@@ -8367,7 +8398,7 @@
     </row>
     <row r="370" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A370" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B370" s="1" t="n">
         <v>9</v>
@@ -8381,7 +8412,7 @@
     </row>
     <row r="371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B371" s="1" t="n">
         <v>10</v>
@@ -8395,7 +8426,7 @@
     </row>
     <row r="372" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B372" s="1" t="n">
         <v>11</v>
@@ -8409,7 +8440,7 @@
     </row>
     <row r="373" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B373" s="1" t="n">
         <v>12</v>
@@ -8423,7 +8454,7 @@
     </row>
     <row r="374" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B374" s="1" t="n">
         <v>13</v>
@@ -8437,7 +8468,7 @@
     </row>
     <row r="375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A375" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B375" s="1" t="n">
         <v>14</v>
@@ -8451,7 +8482,7 @@
     </row>
     <row r="376" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B376" s="1" t="n">
         <v>1</v>
@@ -8465,7 +8496,7 @@
     </row>
     <row r="377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A377" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B377" s="1" t="n">
         <v>2</v>
@@ -8479,7 +8510,7 @@
     </row>
     <row r="378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A378" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B378" s="1" t="n">
         <v>3</v>
@@ -8493,7 +8524,7 @@
     </row>
     <row r="379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A379" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B379" s="1" t="n">
         <v>4</v>
@@ -8507,7 +8538,7 @@
     </row>
     <row r="380" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A380" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B380" s="1" t="n">
         <v>5</v>
@@ -8521,7 +8552,7 @@
     </row>
     <row r="381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B381" s="1" t="n">
         <v>6</v>
@@ -8535,7 +8566,7 @@
     </row>
     <row r="382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A382" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B382" s="1" t="n">
         <v>7</v>
@@ -8549,7 +8580,7 @@
     </row>
     <row r="383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A383" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B383" s="1" t="n">
         <v>8</v>
@@ -8563,7 +8594,7 @@
     </row>
     <row r="384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A384" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B384" s="1" t="n">
         <v>9</v>
@@ -8577,7 +8608,7 @@
     </row>
     <row r="385" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B385" s="1" t="n">
         <v>10</v>
@@ -8591,7 +8622,7 @@
     </row>
     <row r="386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B386" s="1" t="n">
         <v>11</v>
@@ -8605,7 +8636,7 @@
     </row>
     <row r="387" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B387" s="1" t="n">
         <v>12</v>
@@ -8619,7 +8650,7 @@
     </row>
     <row r="388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B388" s="1" t="n">
         <v>13</v>
@@ -8633,7 +8664,7 @@
     </row>
     <row r="389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B389" s="1" t="n">
         <v>14</v>
@@ -8647,7 +8678,7 @@
     </row>
     <row r="390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A390" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B390" s="1" t="n">
         <v>15</v>
@@ -8661,7 +8692,7 @@
     </row>
     <row r="391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A391" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B391" s="1" t="n">
         <v>1</v>
@@ -8675,7 +8706,7 @@
     </row>
     <row r="392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B392" s="1" t="n">
         <v>2</v>
@@ -8689,7 +8720,7 @@
     </row>
     <row r="393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B393" s="1" t="n">
         <v>3</v>
@@ -8703,7 +8734,7 @@
     </row>
     <row r="394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A394" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B394" s="1" t="n">
         <v>4</v>
@@ -8717,7 +8748,7 @@
     </row>
     <row r="395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A395" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B395" s="1" t="n">
         <v>5</v>
@@ -8731,7 +8762,7 @@
     </row>
     <row r="396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A396" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B396" s="1" t="n">
         <v>6</v>
@@ -8745,7 +8776,7 @@
     </row>
     <row r="397" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B397" s="1" t="n">
         <v>7</v>
@@ -8759,7 +8790,7 @@
     </row>
     <row r="398" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B398" s="1" t="n">
         <v>8</v>
@@ -8773,7 +8804,7 @@
     </row>
     <row r="399" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A399" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B399" s="1" t="n">
         <v>1</v>
@@ -8787,7 +8818,7 @@
     </row>
     <row r="400" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A400" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B400" s="1" t="n">
         <v>2</v>
@@ -8801,7 +8832,7 @@
     </row>
     <row r="401" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A401" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B401" s="1" t="n">
         <v>3</v>
@@ -8815,7 +8846,7 @@
     </row>
     <row r="402" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B402" s="1" t="n">
         <v>4</v>
@@ -8829,7 +8860,7 @@
     </row>
     <row r="403" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A403" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B403" s="1" t="n">
         <v>5</v>
@@ -8843,7 +8874,7 @@
     </row>
     <row r="404" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A404" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B404" s="1" t="n">
         <v>6</v>
@@ -8857,7 +8888,7 @@
     </row>
     <row r="405" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A405" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B405" s="1" t="n">
         <v>7</v>
@@ -8871,7 +8902,7 @@
     </row>
     <row r="406" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A406" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B406" s="1" t="n">
         <v>8</v>
@@ -8885,7 +8916,7 @@
     </row>
     <row r="407" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A407" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B407" s="1" t="n">
         <v>1</v>
@@ -8899,7 +8930,7 @@
     </row>
     <row r="408" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A408" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B408" s="1" t="n">
         <v>2</v>
@@ -8913,7 +8944,7 @@
     </row>
     <row r="409" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A409" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B409" s="1" t="n">
         <v>3</v>
@@ -8927,7 +8958,7 @@
     </row>
     <row r="410" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B410" s="1" t="n">
         <v>4</v>
@@ -8941,7 +8972,7 @@
     </row>
     <row r="411" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B411" s="1" t="n">
         <v>5</v>
@@ -8955,7 +8986,7 @@
     </row>
     <row r="412" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B412" s="1" t="n">
         <v>6</v>
@@ -8969,7 +9000,7 @@
     </row>
     <row r="413" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A413" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B413" s="1" t="n">
         <v>7</v>
@@ -8983,7 +9014,7 @@
     </row>
     <row r="414" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A414" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B414" s="1" t="n">
         <v>8</v>
@@ -8997,7 +9028,7 @@
     </row>
     <row r="415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B415" s="1" t="n">
         <v>1</v>
@@ -9011,7 +9042,7 @@
     </row>
     <row r="416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B416" s="1" t="n">
         <v>2</v>
@@ -9025,7 +9056,7 @@
     </row>
     <row r="417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B417" s="1" t="n">
         <v>3</v>
@@ -9039,7 +9070,7 @@
     </row>
     <row r="418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B418" s="1" t="n">
         <v>4</v>
@@ -9053,7 +9084,7 @@
     </row>
     <row r="419" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A419" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B419" s="1" t="n">
         <v>5</v>
@@ -9067,7 +9098,7 @@
     </row>
     <row r="420" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A420" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B420" s="1" t="n">
         <v>6</v>
@@ -9081,7 +9112,7 @@
     </row>
     <row r="421" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A421" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B421" s="1" t="n">
         <v>7</v>
@@ -9095,7 +9126,7 @@
     </row>
     <row r="422" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A422" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B422" s="1" t="n">
         <v>8</v>
@@ -9109,7 +9140,7 @@
     </row>
     <row r="423" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A423" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B423" s="1" t="n">
         <v>9</v>
@@ -9123,7 +9154,7 @@
     </row>
     <row r="424" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A424" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B424" s="1" t="n">
         <v>10</v>
@@ -9137,7 +9168,7 @@
     </row>
     <row r="425" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B425" s="1" t="n">
         <v>11</v>
@@ -9151,7 +9182,7 @@
     </row>
     <row r="426" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A426" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B426" s="1" t="n">
         <v>12</v>
@@ -9165,7 +9196,7 @@
     </row>
     <row r="427" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A427" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B427" s="1" t="n">
         <v>13</v>
@@ -9179,7 +9210,7 @@
     </row>
     <row r="428" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A428" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B428" s="1" t="n">
         <v>14</v>
@@ -9193,7 +9224,7 @@
     </row>
     <row r="429" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A429" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B429" s="1" t="n">
         <v>15</v>
@@ -9207,7 +9238,7 @@
     </row>
     <row r="430" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A430" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B430" s="1" t="n">
         <v>1</v>
@@ -9221,7 +9252,7 @@
     </row>
     <row r="431" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B431" s="1" t="n">
         <v>2</v>
@@ -9235,7 +9266,7 @@
     </row>
     <row r="432" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A432" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B432" s="1" t="n">
         <v>3</v>
@@ -9249,7 +9280,7 @@
     </row>
     <row r="433" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A433" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B433" s="1" t="n">
         <v>4</v>
@@ -9263,7 +9294,7 @@
     </row>
     <row r="434" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A434" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B434" s="1" t="n">
         <v>5</v>
@@ -9277,7 +9308,7 @@
     </row>
     <row r="435" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A435" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B435" s="1" t="n">
         <v>6</v>
@@ -9291,7 +9322,7 @@
     </row>
     <row r="436" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A436" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B436" s="1" t="n">
         <v>7</v>
@@ -9305,7 +9336,7 @@
     </row>
     <row r="437" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A437" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B437" s="1" t="n">
         <v>8</v>
@@ -9319,7 +9350,7 @@
     </row>
     <row r="438" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A438" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B438" s="1" t="n">
         <v>9</v>
@@ -9333,7 +9364,7 @@
     </row>
     <row r="439" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A439" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B439" s="1" t="n">
         <v>10</v>
@@ -9347,7 +9378,7 @@
     </row>
     <row r="440" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A440" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B440" s="1" t="n">
         <v>11</v>
@@ -9361,7 +9392,7 @@
     </row>
     <row r="441" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A441" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B441" s="1" t="n">
         <v>12</v>
@@ -9375,7 +9406,7 @@
     </row>
     <row r="442" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A442" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B442" s="1" t="n">
         <v>13</v>
@@ -9389,7 +9420,7 @@
     </row>
     <row r="443" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A443" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B443" s="1" t="n">
         <v>14</v>
@@ -9403,7 +9434,7 @@
     </row>
     <row r="444" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A444" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B444" s="1" t="n">
         <v>15</v>
@@ -9417,7 +9448,7 @@
     </row>
     <row r="445" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B445" s="1" t="n">
         <v>1</v>
@@ -9431,7 +9462,7 @@
     </row>
     <row r="446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B446" s="1" t="n">
         <v>2</v>
@@ -9445,7 +9476,7 @@
     </row>
     <row r="447" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A447" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B447" s="1" t="n">
         <v>3</v>
@@ -9459,7 +9490,7 @@
     </row>
     <row r="448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A448" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B448" s="1" t="n">
         <v>4</v>
@@ -9473,7 +9504,7 @@
     </row>
     <row r="449" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B449" s="1" t="n">
         <v>5</v>
@@ -9487,7 +9518,7 @@
     </row>
     <row r="450" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A450" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B450" s="1" t="n">
         <v>6</v>
@@ -9501,7 +9532,7 @@
     </row>
     <row r="451" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A451" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B451" s="1" t="n">
         <v>7</v>
@@ -9515,7 +9546,7 @@
     </row>
     <row r="452" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A452" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B452" s="1" t="n">
         <v>8</v>
@@ -9529,7 +9560,7 @@
     </row>
     <row r="453" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A453" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B453" s="1" t="n">
         <v>9</v>
@@ -9543,7 +9574,7 @@
     </row>
     <row r="454" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A454" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B454" s="1" t="n">
         <v>10</v>
@@ -9557,7 +9588,7 @@
     </row>
     <row r="455" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A455" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B455" s="1" t="n">
         <v>11</v>
@@ -9571,7 +9602,7 @@
     </row>
     <row r="456" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A456" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B456" s="1" t="n">
         <v>12</v>
@@ -9585,7 +9616,7 @@
     </row>
     <row r="457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A457" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B457" s="1" t="n">
         <v>13</v>
@@ -9599,7 +9630,7 @@
     </row>
     <row r="458" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A458" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B458" s="1" t="n">
         <v>14</v>
@@ -9613,7 +9644,7 @@
     </row>
     <row r="459" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A459" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B459" s="1" t="n">
         <v>15</v>
@@ -9627,7 +9658,7 @@
     </row>
     <row r="460" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A460" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B460" s="1" t="n">
         <v>1</v>
@@ -9641,7 +9672,7 @@
     </row>
     <row r="461" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A461" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B461" s="1" t="n">
         <v>2</v>
@@ -9655,7 +9686,7 @@
     </row>
     <row r="462" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A462" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B462" s="1" t="n">
         <v>3</v>
@@ -9669,7 +9700,7 @@
     </row>
     <row r="463" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A463" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B463" s="1" t="n">
         <v>4</v>
@@ -9683,7 +9714,7 @@
     </row>
     <row r="464" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A464" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B464" s="1" t="n">
         <v>5</v>
@@ -9697,7 +9728,7 @@
     </row>
     <row r="465" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B465" s="1" t="n">
         <v>6</v>
@@ -9711,7 +9742,7 @@
     </row>
     <row r="466" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A466" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B466" s="1" t="n">
         <v>7</v>
@@ -9725,7 +9756,7 @@
     </row>
     <row r="467" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A467" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B467" s="1" t="n">
         <v>8</v>
@@ -9739,7 +9770,7 @@
     </row>
     <row r="468" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A468" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B468" s="1" t="n">
         <v>9</v>
@@ -9753,7 +9784,7 @@
     </row>
     <row r="469" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A469" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B469" s="1" t="n">
         <v>10</v>
@@ -9767,7 +9798,7 @@
     </row>
     <row r="470" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A470" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B470" s="1" t="n">
         <v>11</v>
@@ -9781,7 +9812,7 @@
     </row>
     <row r="471" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A471" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B471" s="1" t="n">
         <v>12</v>
@@ -9795,7 +9826,7 @@
     </row>
     <row r="472" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A472" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B472" s="1" t="n">
         <v>13</v>
@@ -9809,7 +9840,7 @@
     </row>
     <row r="473" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A473" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B473" s="1" t="n">
         <v>14</v>
@@ -9823,7 +9854,7 @@
     </row>
     <row r="474" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A474" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B474" s="1" t="n">
         <v>15</v>
@@ -9837,7 +9868,7 @@
     </row>
     <row r="475" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A475" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B475" s="1" t="n">
         <v>1</v>
@@ -9851,7 +9882,7 @@
     </row>
     <row r="476" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A476" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B476" s="1" t="n">
         <v>2</v>
@@ -9865,7 +9896,7 @@
     </row>
     <row r="477" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A477" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B477" s="1" t="n">
         <v>3</v>
@@ -9879,7 +9910,7 @@
     </row>
     <row r="478" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A478" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B478" s="1" t="n">
         <v>4</v>
@@ -9893,7 +9924,7 @@
     </row>
     <row r="479" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A479" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B479" s="1" t="n">
         <v>5</v>
@@ -9907,7 +9938,7 @@
     </row>
     <row r="480" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A480" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B480" s="1" t="n">
         <v>6</v>
@@ -9921,7 +9952,7 @@
     </row>
     <row r="481" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A481" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B481" s="1" t="n">
         <v>7</v>
@@ -9935,7 +9966,7 @@
     </row>
     <row r="482" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A482" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B482" s="1" t="n">
         <v>8</v>
@@ -9949,7 +9980,7 @@
     </row>
     <row r="483" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A483" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B483" s="1" t="n">
         <v>9</v>
@@ -9963,7 +9994,7 @@
     </row>
     <row r="484" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A484" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B484" s="1" t="n">
         <v>10</v>
@@ -9977,7 +10008,7 @@
     </row>
     <row r="485" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A485" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B485" s="1" t="n">
         <v>11</v>
@@ -9991,7 +10022,7 @@
     </row>
     <row r="486" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A486" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B486" s="1" t="n">
         <v>12</v>
@@ -10005,7 +10036,7 @@
     </row>
     <row r="487" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A487" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B487" s="1" t="n">
         <v>13</v>
@@ -10019,7 +10050,7 @@
     </row>
     <row r="488" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A488" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B488" s="1" t="n">
         <v>14</v>
@@ -10033,7 +10064,7 @@
     </row>
     <row r="489" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A489" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B489" s="1" t="n">
         <v>15</v>
@@ -10047,7 +10078,7 @@
     </row>
     <row r="490" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A490" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B490" s="1" t="n">
         <v>1</v>
@@ -10061,7 +10092,7 @@
     </row>
     <row r="491" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A491" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B491" s="1" t="n">
         <v>2</v>
@@ -10075,7 +10106,7 @@
     </row>
     <row r="492" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A492" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B492" s="1" t="n">
         <v>3</v>
@@ -10089,7 +10120,7 @@
     </row>
     <row r="493" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A493" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B493" s="1" t="n">
         <v>4</v>
@@ -10103,7 +10134,7 @@
     </row>
     <row r="494" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A494" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B494" s="1" t="n">
         <v>5</v>
@@ -10117,7 +10148,7 @@
     </row>
     <row r="495" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A495" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B495" s="1" t="n">
         <v>6</v>
@@ -10131,7 +10162,7 @@
     </row>
     <row r="496" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A496" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B496" s="1" t="n">
         <v>7</v>
@@ -10145,7 +10176,7 @@
     </row>
     <row r="497" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A497" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B497" s="1" t="n">
         <v>8</v>
@@ -10159,7 +10190,7 @@
     </row>
     <row r="498" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A498" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B498" s="1" t="n">
         <v>9</v>
@@ -10173,7 +10204,7 @@
     </row>
     <row r="499" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A499" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B499" s="1" t="n">
         <v>10</v>
@@ -10187,7 +10218,7 @@
     </row>
     <row r="500" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A500" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B500" s="1" t="n">
         <v>11</v>
@@ -10201,7 +10232,7 @@
     </row>
     <row r="501" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A501" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B501" s="1" t="n">
         <v>12</v>
@@ -10215,7 +10246,7 @@
     </row>
     <row r="502" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A502" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B502" s="1" t="n">
         <v>13</v>
@@ -10229,7 +10260,7 @@
     </row>
     <row r="503" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A503" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B503" s="1" t="n">
         <v>14</v>
@@ -10243,7 +10274,7 @@
     </row>
     <row r="504" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A504" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B504" s="1" t="n">
         <v>15</v>

</xml_diff>

<commit_message>
2025 Yılı Maaş Kat Sayıları eklendi.
</commit_message>
<xml_diff>
--- a/maas_verileri.xlsx
+++ b/maas_verileri.xlsx
@@ -8,10 +8,10 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="maas_kat_sayilari" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="yan_odeme_puanlari" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="ozel_hizmet_tazminati" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="maas_kat_sayilari" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="yan_odeme_puanlari" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="ozel_hizmet_tazminati" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -351,6 +351,112 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -816,7 +922,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="10.46"/>
@@ -1397,6 +1503,20 @@
       </c>
       <c r="D41" s="2" t="n">
         <v>14.208727</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="n">
+        <v>45658</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>1.012556</v>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>0.321115</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>15.848415</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Yeni bir sayfa eklendi.
</commit_message>
<xml_diff>
--- a/maas_verileri.xlsx
+++ b/maas_verileri.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId3"/>
@@ -355,7 +355,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -401,10 +401,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9854,262 +9850,262 @@
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="18.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="12" width="28.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="12" width="19.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="12" width="13.81"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="12" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.8"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="1" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="n">
+      <c r="A2" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="n">
+      <c r="A3" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="1" t="n">
         <v>62</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="1" t="n">
         <v>68</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="n">
-        <v>70</v>
-      </c>
-      <c r="B7" s="12" t="s">
+      <c r="A7" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="1" t="n">
         <v>71</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="1" t="n">
         <v>73</v>
       </c>
-      <c r="B9" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="C9" s="12" t="s">
+      <c r="B9" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="1" t="n">
         <v>107</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="n">
+      <c r="A11" s="1" t="n">
         <v>114</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="1" t="n">
         <v>115</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="n">
+      <c r="A13" s="1" t="n">
         <v>116</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="1" t="n">
         <v>127</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="1" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="n">
+      <c r="A15" s="1" t="n">
         <v>129</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="1" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="n">
+      <c r="A16" s="1" t="n">
         <v>137</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="1" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="1" t="n">
         <v>155</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="1" t="n">
         <v>367</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="1" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
kadro Ünvan Sıra No için yeni ünvanlar eklendi.
</commit_message>
<xml_diff>
--- a/maas_verileri.xlsx
+++ b/maas_verileri.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="87">
   <si>
     <t xml:space="preserve">yil</t>
   </si>
@@ -212,6 +212,9 @@
     <t xml:space="preserve">personel_tipi</t>
   </si>
   <si>
+    <t xml:space="preserve">İl Müftü Yardımcısı</t>
+  </si>
+  <si>
     <t xml:space="preserve">İlçe Müftüsü</t>
   </si>
   <si>
@@ -227,7 +230,19 @@
     <t xml:space="preserve">Din Hizmetleri</t>
   </si>
   <si>
+    <t xml:space="preserve">Uzman Vaiz - Alo Fetva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cezaevi Vaizi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kuran Kursu Uzm. Öğrt.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kuran Kursu Öğreticisi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baş İmam Hatip</t>
   </si>
   <si>
     <t xml:space="preserve">Uzman İmam Hatip</t>
@@ -243,6 +258,9 @@
   </si>
   <si>
     <t xml:space="preserve">Yardımcı Hizmetler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaloriferci</t>
   </si>
   <si>
     <t xml:space="preserve">4/B M.K.</t>
@@ -358,7 +376,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -407,6 +425,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,6 +438,15 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -9850,7 +9881,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.68"/>
@@ -9876,13 +9907,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>63</v>
+        <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>32</v>
@@ -9890,13 +9918,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>32</v>
@@ -9904,13 +9929,13 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>32</v>
@@ -9918,13 +9943,13 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>32</v>
@@ -9932,13 +9957,13 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>32</v>
@@ -9946,41 +9971,37 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>66</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="C7" s="12"/>
       <c r="D7" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>66</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="C8" s="12"/>
       <c r="D8" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>66</v>
+        <v>27</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>67</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>32</v>
@@ -9988,13 +10009,13 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
-        <v>107</v>
+        <v>61</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>67</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>32</v>
@@ -10002,13 +10023,13 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
-        <v>114</v>
+        <v>62</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>32</v>
@@ -10016,13 +10037,13 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
-        <v>115</v>
+        <v>63</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>32</v>
@@ -10030,13 +10051,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
-        <v>116</v>
+        <v>65</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>72</v>
+        <v>25</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>67</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>32</v>
@@ -10044,69 +10065,69 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
-        <v>127</v>
+        <v>67</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>67</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>75</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
-        <v>128</v>
+        <v>68</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>75</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
-        <v>129</v>
+        <v>69</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>75</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
-        <v>137</v>
+        <v>70</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>75</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
-        <v>155</v>
+        <v>71</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>32</v>
@@ -10114,17 +10135,261 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
+        <v>73</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="n">
+        <v>101</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="12"/>
+      <c r="D21" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="n">
+        <v>103</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="12"/>
+      <c r="D22" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="n">
+        <v>107</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="n">
+        <v>114</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="n">
+        <v>115</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="n">
+        <v>116</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="n">
+        <v>117</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="n">
+        <v>118</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="n">
+        <v>119</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="n">
+        <v>127</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="n">
+        <v>128</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="n">
+        <v>129</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="n">
+        <v>137</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="n">
+        <v>155</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="n">
         <v>367</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B35" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>75</v>
-      </c>
+      <c r="D35" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="0"/>
+      <c r="C36" s="12"/>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="0"/>
+      <c r="C37" s="12"/>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="0"/>
+      <c r="C38" s="12"/>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="0"/>
+      <c r="C39" s="12"/>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="0"/>
+      <c r="C40" s="12"/>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="0"/>
+      <c r="C41" s="12"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
@yahyayildirim, bazı önemli değişiklikler yapıldı.
</commit_message>
<xml_diff>
--- a/maas_verileri.xlsx
+++ b/maas_verileri.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="120">
   <si>
     <t xml:space="preserve">yil</t>
   </si>
@@ -174,7 +174,10 @@
     <t xml:space="preserve">Kaloriferc</t>
   </si>
   <si>
-    <t xml:space="preserve">Vekil</t>
+    <t xml:space="preserve">Vekil İ-H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vekil M-K</t>
   </si>
   <si>
     <t xml:space="preserve">oht_orani</t>
@@ -2602,8 +2605,15 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
+      <c r="A65" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B65" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" s="1" t="n">
+        <v>500</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="2"/>
@@ -2667,7 +2677,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M465"/>
+  <dimension ref="A1:M510"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="14.74"/>
@@ -2688,16 +2698,16 @@
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3768,7 +3778,7 @@
         <v>50</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3788,7 +3798,7 @@
         <v>50</v>
       </c>
       <c r="F78" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3808,7 +3818,7 @@
         <v>40</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3828,7 +3838,7 @@
         <v>40</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3848,7 +3858,7 @@
         <v>40</v>
       </c>
       <c r="F81" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3868,7 +3878,7 @@
         <v>25</v>
       </c>
       <c r="F82" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3888,7 +3898,7 @@
         <v>25</v>
       </c>
       <c r="F83" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3908,7 +3918,7 @@
         <v>20</v>
       </c>
       <c r="F84" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3928,7 +3938,7 @@
         <v>20</v>
       </c>
       <c r="F85" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3948,7 +3958,7 @@
         <v>20</v>
       </c>
       <c r="F86" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3965,7 +3975,7 @@
         <v>66</v>
       </c>
       <c r="F87" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3982,7 +3992,7 @@
         <v>66</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3999,7 +4009,7 @@
         <v>66</v>
       </c>
       <c r="F89" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4016,7 +4026,7 @@
         <v>66</v>
       </c>
       <c r="F90" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4033,7 +4043,7 @@
         <v>66</v>
       </c>
       <c r="F91" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4050,7 +4060,7 @@
         <v>66</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4067,7 +4077,7 @@
         <v>66</v>
       </c>
       <c r="F93" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4084,7 +4094,7 @@
         <v>66</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4101,7 +4111,7 @@
         <v>66</v>
       </c>
       <c r="F95" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4118,7 +4128,7 @@
         <v>66</v>
       </c>
       <c r="F96" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4135,7 +4145,7 @@
         <v>66</v>
       </c>
       <c r="F97" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4152,7 +4162,7 @@
         <v>66</v>
       </c>
       <c r="F98" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4169,7 +4179,7 @@
         <v>66</v>
       </c>
       <c r="F99" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4186,7 +4196,7 @@
         <v>66</v>
       </c>
       <c r="F100" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4203,7 +4213,7 @@
         <v>115</v>
       </c>
       <c r="F101" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4220,7 +4230,7 @@
         <v>115</v>
       </c>
       <c r="F102" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4237,7 +4247,7 @@
         <v>105</v>
       </c>
       <c r="F103" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4254,7 +4264,7 @@
         <v>105</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4271,7 +4281,7 @@
         <v>95</v>
       </c>
       <c r="F105" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4288,7 +4298,7 @@
         <v>95</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4305,7 +4315,7 @@
         <v>95</v>
       </c>
       <c r="F107" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4322,7 +4332,7 @@
         <v>90</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4339,7 +4349,7 @@
         <v>90</v>
       </c>
       <c r="F109" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4356,7 +4366,7 @@
         <v>90</v>
       </c>
       <c r="F110" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4373,7 +4383,7 @@
         <v>115</v>
       </c>
       <c r="F111" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4390,7 +4400,7 @@
         <v>115</v>
       </c>
       <c r="F112" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4407,7 +4417,7 @@
         <v>105</v>
       </c>
       <c r="F113" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4424,7 +4434,7 @@
         <v>105</v>
       </c>
       <c r="F114" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4441,7 +4451,7 @@
         <v>95</v>
       </c>
       <c r="F115" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4458,7 +4468,7 @@
         <v>95</v>
       </c>
       <c r="F116" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4475,7 +4485,7 @@
         <v>95</v>
       </c>
       <c r="F117" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4492,7 +4502,7 @@
         <v>90</v>
       </c>
       <c r="F118" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4509,7 +4519,7 @@
         <v>90</v>
       </c>
       <c r="F119" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4526,7 +4536,7 @@
         <v>90</v>
       </c>
       <c r="F120" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4543,7 +4553,7 @@
         <v>115</v>
       </c>
       <c r="F121" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4560,7 +4570,7 @@
         <v>115</v>
       </c>
       <c r="F122" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4577,7 +4587,7 @@
         <v>105</v>
       </c>
       <c r="F123" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4594,7 +4604,7 @@
         <v>105</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4611,7 +4621,7 @@
         <v>95</v>
       </c>
       <c r="F125" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4628,7 +4638,7 @@
         <v>95</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4645,7 +4655,7 @@
         <v>95</v>
       </c>
       <c r="F127" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4662,7 +4672,7 @@
         <v>90</v>
       </c>
       <c r="F128" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4679,7 +4689,7 @@
         <v>90</v>
       </c>
       <c r="F129" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4696,7 +4706,7 @@
         <v>90</v>
       </c>
       <c r="F130" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4713,7 +4723,7 @@
         <v>115</v>
       </c>
       <c r="F131" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4730,7 +4740,7 @@
         <v>115</v>
       </c>
       <c r="F132" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4747,7 +4757,7 @@
         <v>105</v>
       </c>
       <c r="F133" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4764,7 +4774,7 @@
         <v>105</v>
       </c>
       <c r="F134" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4781,7 +4791,7 @@
         <v>95</v>
       </c>
       <c r="F135" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4798,7 +4808,7 @@
         <v>95</v>
       </c>
       <c r="F136" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4815,7 +4825,7 @@
         <v>95</v>
       </c>
       <c r="F137" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4832,7 +4842,7 @@
         <v>90</v>
       </c>
       <c r="F138" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4849,7 +4859,7 @@
         <v>90</v>
       </c>
       <c r="F139" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4866,7 +4876,7 @@
         <v>90</v>
       </c>
       <c r="F140" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4883,7 +4893,7 @@
         <v>65</v>
       </c>
       <c r="F141" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4900,7 +4910,7 @@
         <v>65</v>
       </c>
       <c r="F142" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4917,7 +4927,7 @@
         <v>65</v>
       </c>
       <c r="F143" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4934,7 +4944,7 @@
         <v>65</v>
       </c>
       <c r="F144" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4951,7 +4961,7 @@
         <v>65</v>
       </c>
       <c r="F145" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4968,7 +4978,7 @@
         <v>65</v>
       </c>
       <c r="F146" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4985,7 +4995,7 @@
         <v>65</v>
       </c>
       <c r="F147" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5002,7 +5012,7 @@
         <v>65</v>
       </c>
       <c r="F148" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5019,7 +5029,7 @@
         <v>65</v>
       </c>
       <c r="F149" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5036,7 +5046,7 @@
         <v>65</v>
       </c>
       <c r="F150" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5053,7 +5063,7 @@
         <v>65</v>
       </c>
       <c r="F151" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5070,7 +5080,7 @@
         <v>65</v>
       </c>
       <c r="F152" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5087,7 +5097,7 @@
         <v>65</v>
       </c>
       <c r="F153" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5104,7 +5114,7 @@
         <v>65</v>
       </c>
       <c r="F154" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5121,7 +5131,7 @@
         <v>65</v>
       </c>
       <c r="F155" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5138,7 +5148,7 @@
         <v>65</v>
       </c>
       <c r="F156" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5155,7 +5165,7 @@
         <v>65</v>
       </c>
       <c r="F157" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5172,7 +5182,7 @@
         <v>65</v>
       </c>
       <c r="F158" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5189,7 +5199,7 @@
         <v>65</v>
       </c>
       <c r="F159" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5206,7 +5216,7 @@
         <v>65</v>
       </c>
       <c r="F160" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5226,7 +5236,7 @@
         <v>50</v>
       </c>
       <c r="F161" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5246,7 +5256,7 @@
         <v>50</v>
       </c>
       <c r="F162" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5266,7 +5276,7 @@
         <v>40</v>
       </c>
       <c r="F163" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5286,7 +5296,7 @@
         <v>40</v>
       </c>
       <c r="F164" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5306,7 +5316,7 @@
         <v>25</v>
       </c>
       <c r="F165" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5326,7 +5336,7 @@
         <v>25</v>
       </c>
       <c r="F166" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5346,7 +5356,7 @@
         <v>20</v>
       </c>
       <c r="F167" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5366,7 +5376,7 @@
         <v>20</v>
       </c>
       <c r="F168" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5386,7 +5396,7 @@
         <v>20</v>
       </c>
       <c r="F169" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5406,7 +5416,7 @@
         <v>20</v>
       </c>
       <c r="F170" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5423,7 +5433,7 @@
         <v>70</v>
       </c>
       <c r="F171" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5440,7 +5450,7 @@
         <v>70</v>
       </c>
       <c r="F172" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5457,7 +5467,7 @@
         <v>70</v>
       </c>
       <c r="F173" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5474,7 +5484,7 @@
         <v>70</v>
       </c>
       <c r="F174" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5491,7 +5501,7 @@
         <v>70</v>
       </c>
       <c r="F175" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5508,7 +5518,7 @@
         <v>70</v>
       </c>
       <c r="F176" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5525,7 +5535,7 @@
         <v>70</v>
       </c>
       <c r="F177" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5542,7 +5552,7 @@
         <v>70</v>
       </c>
       <c r="F178" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5559,7 +5569,7 @@
         <v>70</v>
       </c>
       <c r="F179" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5576,7 +5586,7 @@
         <v>70</v>
       </c>
       <c r="F180" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5593,7 +5603,7 @@
         <v>70</v>
       </c>
       <c r="F181" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5610,7 +5620,7 @@
         <v>70</v>
       </c>
       <c r="F182" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5627,7 +5637,7 @@
         <v>70</v>
       </c>
       <c r="F183" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5644,7 +5654,7 @@
         <v>70</v>
       </c>
       <c r="F184" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5661,7 +5671,7 @@
         <v>70</v>
       </c>
       <c r="F185" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5678,7 +5688,7 @@
         <v>70</v>
       </c>
       <c r="F186" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5695,7 +5705,7 @@
         <v>70</v>
       </c>
       <c r="F187" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5712,7 +5722,7 @@
         <v>70</v>
       </c>
       <c r="F188" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5729,7 +5739,7 @@
         <v>70</v>
       </c>
       <c r="F189" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5746,7 +5756,7 @@
         <v>70</v>
       </c>
       <c r="F190" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5763,7 +5773,7 @@
         <v>70</v>
       </c>
       <c r="F191" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5780,7 +5790,7 @@
         <v>70</v>
       </c>
       <c r="F192" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5797,7 +5807,7 @@
         <v>70</v>
       </c>
       <c r="F193" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5814,7 +5824,7 @@
         <v>70</v>
       </c>
       <c r="F194" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5831,7 +5841,7 @@
         <v>70</v>
       </c>
       <c r="F195" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5848,7 +5858,7 @@
         <v>70</v>
       </c>
       <c r="F196" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5865,7 +5875,7 @@
         <v>70</v>
       </c>
       <c r="F197" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5882,7 +5892,7 @@
         <v>70</v>
       </c>
       <c r="F198" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5899,7 +5909,7 @@
         <v>70</v>
       </c>
       <c r="F199" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5916,7 +5926,7 @@
         <v>70</v>
       </c>
       <c r="F200" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5933,7 +5943,7 @@
         <v>70</v>
       </c>
       <c r="F201" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5950,7 +5960,7 @@
         <v>70</v>
       </c>
       <c r="F202" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5967,7 +5977,7 @@
         <v>70</v>
       </c>
       <c r="F203" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5984,7 +5994,7 @@
         <v>70</v>
       </c>
       <c r="F204" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6001,7 +6011,7 @@
         <v>70</v>
       </c>
       <c r="F205" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6018,7 +6028,7 @@
         <v>70</v>
       </c>
       <c r="F206" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6035,7 +6045,7 @@
         <v>70</v>
       </c>
       <c r="F207" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6052,7 +6062,7 @@
         <v>70</v>
       </c>
       <c r="F208" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6069,7 +6079,7 @@
         <v>70</v>
       </c>
       <c r="F209" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6086,7 +6096,7 @@
         <v>70</v>
       </c>
       <c r="F210" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6103,7 +6113,7 @@
         <v>70</v>
       </c>
       <c r="F211" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6120,7 +6130,7 @@
         <v>70</v>
       </c>
       <c r="F212" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6137,7 +6147,7 @@
         <v>70</v>
       </c>
       <c r="F213" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6154,7 +6164,7 @@
         <v>70</v>
       </c>
       <c r="F214" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6171,7 +6181,7 @@
         <v>70</v>
       </c>
       <c r="F215" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6191,7 +6201,7 @@
         <v>25</v>
       </c>
       <c r="F216" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6211,7 +6221,7 @@
         <v>25</v>
       </c>
       <c r="F217" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6231,7 +6241,7 @@
         <v>20</v>
       </c>
       <c r="F218" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6251,7 +6261,7 @@
         <v>20</v>
       </c>
       <c r="F219" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6268,7 +6278,7 @@
         <v>70</v>
       </c>
       <c r="F220" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6285,7 +6295,7 @@
         <v>70</v>
       </c>
       <c r="F221" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6302,7 +6312,7 @@
         <v>70</v>
       </c>
       <c r="F222" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6319,7 +6329,7 @@
         <v>70</v>
       </c>
       <c r="F223" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6336,7 +6346,7 @@
         <v>70</v>
       </c>
       <c r="F224" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6353,7 +6363,7 @@
         <v>70</v>
       </c>
       <c r="F225" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6370,7 +6380,7 @@
         <v>70</v>
       </c>
       <c r="F226" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6387,7 +6397,7 @@
         <v>70</v>
       </c>
       <c r="F227" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6404,7 +6414,7 @@
         <v>70</v>
       </c>
       <c r="F228" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6421,7 +6431,7 @@
         <v>70</v>
       </c>
       <c r="F229" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6438,7 +6448,7 @@
         <v>70</v>
       </c>
       <c r="F230" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6455,7 +6465,7 @@
         <v>70</v>
       </c>
       <c r="F231" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6472,7 +6482,7 @@
         <v>70</v>
       </c>
       <c r="F232" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6489,7 +6499,7 @@
         <v>70</v>
       </c>
       <c r="F233" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6506,7 +6516,7 @@
         <v>70</v>
       </c>
       <c r="F234" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6523,7 +6533,7 @@
         <v>70</v>
       </c>
       <c r="F235" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6540,7 +6550,7 @@
         <v>70</v>
       </c>
       <c r="F236" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6557,7 +6567,7 @@
         <v>70</v>
       </c>
       <c r="F237" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6574,7 +6584,7 @@
         <v>70</v>
       </c>
       <c r="F238" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6591,7 +6601,7 @@
         <v>70</v>
       </c>
       <c r="F239" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6608,7 +6618,7 @@
         <v>70</v>
       </c>
       <c r="F240" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6625,7 +6635,7 @@
         <v>70</v>
       </c>
       <c r="F241" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6642,7 +6652,7 @@
         <v>70</v>
       </c>
       <c r="F242" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6659,7 +6669,7 @@
         <v>70</v>
       </c>
       <c r="F243" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6676,7 +6686,7 @@
         <v>70</v>
       </c>
       <c r="F244" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6693,7 +6703,7 @@
         <v>70</v>
       </c>
       <c r="F245" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6710,7 +6720,7 @@
         <v>70</v>
       </c>
       <c r="F246" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6727,7 +6737,7 @@
         <v>70</v>
       </c>
       <c r="F247" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6744,7 +6754,7 @@
         <v>70</v>
       </c>
       <c r="F248" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6761,7 +6771,7 @@
         <v>70</v>
       </c>
       <c r="F249" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="250" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6778,7 +6788,7 @@
         <v>70</v>
       </c>
       <c r="F250" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6795,7 +6805,7 @@
         <v>70</v>
       </c>
       <c r="F251" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6812,7 +6822,7 @@
         <v>70</v>
       </c>
       <c r="F252" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6829,7 +6839,7 @@
         <v>70</v>
       </c>
       <c r="F253" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6846,7 +6856,7 @@
         <v>70</v>
       </c>
       <c r="F254" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6863,7 +6873,7 @@
         <v>70</v>
       </c>
       <c r="F255" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6880,7 +6890,7 @@
         <v>70</v>
       </c>
       <c r="F256" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="257" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6897,7 +6907,7 @@
         <v>70</v>
       </c>
       <c r="F257" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6914,7 +6924,7 @@
         <v>70</v>
       </c>
       <c r="F258" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6931,7 +6941,7 @@
         <v>70</v>
       </c>
       <c r="F259" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6948,7 +6958,7 @@
         <v>70</v>
       </c>
       <c r="F260" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="261" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6965,7 +6975,7 @@
         <v>70</v>
       </c>
       <c r="F261" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6982,7 +6992,7 @@
         <v>70</v>
       </c>
       <c r="F262" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="263" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6999,7 +7009,7 @@
         <v>70</v>
       </c>
       <c r="F263" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="264" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7016,7 +7026,7 @@
         <v>70</v>
       </c>
       <c r="F264" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7036,7 +7046,7 @@
         <v>50</v>
       </c>
       <c r="F265" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7056,7 +7066,7 @@
         <v>50</v>
       </c>
       <c r="F266" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7076,7 +7086,7 @@
         <v>40</v>
       </c>
       <c r="F267" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7096,7 +7106,7 @@
         <v>40</v>
       </c>
       <c r="F268" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="269" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7116,7 +7126,7 @@
         <v>25</v>
       </c>
       <c r="F269" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="270" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7136,7 +7146,7 @@
         <v>25</v>
       </c>
       <c r="F270" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="271" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7156,7 +7166,7 @@
         <v>20</v>
       </c>
       <c r="F271" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7176,7 +7186,7 @@
         <v>20</v>
       </c>
       <c r="F272" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7196,7 +7206,7 @@
         <v>20</v>
       </c>
       <c r="F273" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7216,7 +7226,7 @@
         <v>20</v>
       </c>
       <c r="F274" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7236,7 +7246,7 @@
         <v>20</v>
       </c>
       <c r="F275" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7256,7 +7266,7 @@
         <v>20</v>
       </c>
       <c r="F276" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7273,7 +7283,7 @@
         <v>65</v>
       </c>
       <c r="F277" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7290,7 +7300,7 @@
         <v>65</v>
       </c>
       <c r="F278" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7307,7 +7317,7 @@
         <v>65</v>
       </c>
       <c r="F279" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7324,7 +7334,7 @@
         <v>65</v>
       </c>
       <c r="F280" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7341,7 +7351,7 @@
         <v>65</v>
       </c>
       <c r="F281" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7358,7 +7368,7 @@
         <v>65</v>
       </c>
       <c r="F282" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="283" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7375,7 +7385,7 @@
         <v>65</v>
       </c>
       <c r="F283" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7392,7 +7402,7 @@
         <v>65</v>
       </c>
       <c r="F284" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7409,7 +7419,7 @@
         <v>65</v>
       </c>
       <c r="F285" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7426,7 +7436,7 @@
         <v>65</v>
       </c>
       <c r="F286" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7443,7 +7453,7 @@
         <v>65</v>
       </c>
       <c r="F287" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7460,7 +7470,7 @@
         <v>65</v>
       </c>
       <c r="F288" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7477,7 +7487,7 @@
         <v>65</v>
       </c>
       <c r="F289" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7494,7 +7504,7 @@
         <v>65</v>
       </c>
       <c r="F290" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7511,7 +7521,7 @@
         <v>65</v>
       </c>
       <c r="F291" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7528,7 +7538,7 @@
         <v>65</v>
       </c>
       <c r="F292" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="293" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7545,7 +7555,7 @@
         <v>65</v>
       </c>
       <c r="F293" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="294" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7562,7 +7572,7 @@
         <v>65</v>
       </c>
       <c r="F294" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7579,7 +7589,7 @@
         <v>65</v>
       </c>
       <c r="F295" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="296" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7596,7 +7606,7 @@
         <v>65</v>
       </c>
       <c r="F296" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="297" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7613,7 +7623,7 @@
         <v>65</v>
       </c>
       <c r="F297" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="298" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7630,7 +7640,7 @@
         <v>65</v>
       </c>
       <c r="F298" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="299" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7647,7 +7657,7 @@
         <v>65</v>
       </c>
       <c r="F299" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="300" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7664,7 +7674,7 @@
         <v>65</v>
       </c>
       <c r="F300" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="301" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7681,7 +7691,7 @@
         <v>65</v>
       </c>
       <c r="F301" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="302" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7698,7 +7708,7 @@
         <v>65</v>
       </c>
       <c r="F302" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="303" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7715,7 +7725,7 @@
         <v>65</v>
       </c>
       <c r="F303" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="304" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7732,7 +7742,7 @@
         <v>65</v>
       </c>
       <c r="F304" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="305" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7749,7 +7759,7 @@
         <v>65</v>
       </c>
       <c r="F305" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="306" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7766,7 +7776,7 @@
         <v>65</v>
       </c>
       <c r="F306" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="307" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7783,7 +7793,7 @@
         <v>65</v>
       </c>
       <c r="F307" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="308" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7800,7 +7810,7 @@
         <v>65</v>
       </c>
       <c r="F308" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="309" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7817,7 +7827,7 @@
         <v>65</v>
       </c>
       <c r="F309" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="310" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7834,7 +7844,7 @@
         <v>65</v>
       </c>
       <c r="F310" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="311" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7851,7 +7861,7 @@
         <v>65</v>
       </c>
       <c r="F311" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="312" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7868,7 +7878,7 @@
         <v>65</v>
       </c>
       <c r="F312" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="313" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7885,7 +7895,7 @@
         <v>65</v>
       </c>
       <c r="F313" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="314" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7902,7 +7912,7 @@
         <v>65</v>
       </c>
       <c r="F314" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="315" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7919,7 +7929,7 @@
         <v>65</v>
       </c>
       <c r="F315" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="316" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7936,7 +7946,7 @@
         <v>65</v>
       </c>
       <c r="F316" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="317" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7953,7 +7963,7 @@
         <v>65</v>
       </c>
       <c r="F317" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="318" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7970,7 +7980,7 @@
         <v>65</v>
       </c>
       <c r="F318" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="319" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7987,7 +7997,7 @@
         <v>65</v>
       </c>
       <c r="F319" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="320" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8004,7 +8014,7 @@
         <v>65</v>
       </c>
       <c r="F320" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="321" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8021,7 +8031,7 @@
         <v>65</v>
       </c>
       <c r="F321" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="322" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8404,7 +8414,7 @@
     </row>
     <row r="349" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A349" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B349" s="1" t="n">
         <v>1</v>
@@ -8418,7 +8428,7 @@
     </row>
     <row r="350" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A350" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B350" s="1" t="n">
         <v>2</v>
@@ -8432,7 +8442,7 @@
     </row>
     <row r="351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A351" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B351" s="1" t="n">
         <v>3</v>
@@ -8446,7 +8456,7 @@
     </row>
     <row r="352" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A352" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B352" s="1" t="n">
         <v>4</v>
@@ -8460,7 +8470,7 @@
     </row>
     <row r="353" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A353" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B353" s="1" t="n">
         <v>5</v>
@@ -8474,7 +8484,7 @@
     </row>
     <row r="354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A354" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B354" s="1" t="n">
         <v>6</v>
@@ -8488,7 +8498,7 @@
     </row>
     <row r="355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A355" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B355" s="1" t="n">
         <v>7</v>
@@ -8502,7 +8512,7 @@
     </row>
     <row r="356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A356" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B356" s="1" t="n">
         <v>8</v>
@@ -9421,7 +9431,7 @@
         <v>95</v>
       </c>
       <c r="F421" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M421" s="11"/>
     </row>
@@ -9436,7 +9446,7 @@
         <v>95</v>
       </c>
       <c r="F422" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="423" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9450,7 +9460,7 @@
         <v>95</v>
       </c>
       <c r="F423" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="424" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9464,7 +9474,7 @@
         <v>95</v>
       </c>
       <c r="F424" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="425" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9478,7 +9488,7 @@
         <v>94</v>
       </c>
       <c r="F425" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="426" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9492,7 +9502,7 @@
         <v>94</v>
       </c>
       <c r="F426" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="427" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9506,7 +9516,7 @@
         <v>94</v>
       </c>
       <c r="F427" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="428" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9520,7 +9530,7 @@
         <v>94</v>
       </c>
       <c r="F428" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="429" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9534,7 +9544,7 @@
         <v>94</v>
       </c>
       <c r="F429" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="430" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9548,7 +9558,7 @@
         <v>94</v>
       </c>
       <c r="F430" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="431" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9562,7 +9572,7 @@
         <v>94</v>
       </c>
       <c r="F431" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="432" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9576,7 +9586,7 @@
         <v>94</v>
       </c>
       <c r="F432" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="433" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9590,7 +9600,7 @@
         <v>94</v>
       </c>
       <c r="F433" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="434" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9604,7 +9614,7 @@
         <v>94</v>
       </c>
       <c r="F434" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="435" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9618,7 +9628,7 @@
         <v>94</v>
       </c>
       <c r="F435" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="436" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9632,7 +9642,7 @@
         <v>93</v>
       </c>
       <c r="F436" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="437" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9646,7 +9656,7 @@
         <v>93</v>
       </c>
       <c r="F437" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="438" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9660,7 +9670,7 @@
         <v>93</v>
       </c>
       <c r="F438" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="439" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9674,7 +9684,7 @@
         <v>93</v>
       </c>
       <c r="F439" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="440" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9688,7 +9698,7 @@
         <v>92</v>
       </c>
       <c r="F440" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="441" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9702,7 +9712,7 @@
         <v>92</v>
       </c>
       <c r="F441" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="442" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9716,7 +9726,7 @@
         <v>92</v>
       </c>
       <c r="F442" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="443" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9730,7 +9740,7 @@
         <v>92</v>
       </c>
       <c r="F443" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="444" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9744,7 +9754,7 @@
         <v>92</v>
       </c>
       <c r="F444" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="445" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9758,7 +9768,7 @@
         <v>91</v>
       </c>
       <c r="F445" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9772,7 +9782,7 @@
         <v>91</v>
       </c>
       <c r="F446" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="447" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9786,7 +9796,7 @@
         <v>91</v>
       </c>
       <c r="F447" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9800,7 +9810,7 @@
         <v>91</v>
       </c>
       <c r="F448" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="449" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9814,7 +9824,7 @@
         <v>91</v>
       </c>
       <c r="F449" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="450" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9828,7 +9838,7 @@
         <v>91</v>
       </c>
       <c r="F450" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="451" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9842,7 +9852,7 @@
         <v>89</v>
       </c>
       <c r="F451" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="452" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9856,7 +9866,7 @@
         <v>89</v>
       </c>
       <c r="F452" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="453" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9870,7 +9880,7 @@
         <v>89</v>
       </c>
       <c r="F453" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="454" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9884,7 +9894,7 @@
         <v>89</v>
       </c>
       <c r="F454" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="455" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9898,7 +9908,7 @@
         <v>89</v>
       </c>
       <c r="F455" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="456" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9912,7 +9922,7 @@
         <v>89</v>
       </c>
       <c r="F456" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9926,7 +9936,7 @@
         <v>89</v>
       </c>
       <c r="F457" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="458" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9940,7 +9950,7 @@
         <v>88</v>
       </c>
       <c r="F458" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="459" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9954,7 +9964,7 @@
         <v>88</v>
       </c>
       <c r="F459" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="460" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9968,7 +9978,7 @@
         <v>88</v>
       </c>
       <c r="F460" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="461" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9982,7 +9992,7 @@
         <v>88</v>
       </c>
       <c r="F461" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="462" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9996,7 +10006,7 @@
         <v>88</v>
       </c>
       <c r="F462" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="463" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10010,7 +10020,7 @@
         <v>88</v>
       </c>
       <c r="F463" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="464" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10024,7 +10034,7 @@
         <v>88</v>
       </c>
       <c r="F464" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="465" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10038,7 +10048,637 @@
         <v>88</v>
       </c>
       <c r="F465" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="466" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A466" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B466" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C466" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="F466" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="467" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A467" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B467" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C467" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="F467" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="468" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A468" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B468" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C468" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="F468" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="469" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A469" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B469" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C469" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="F469" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="470" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A470" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B470" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C470" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F470" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="471" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A471" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B471" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C471" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F471" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="472" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A472" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B472" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="C472" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F472" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="473" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A473" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B473" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="C473" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F473" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="474" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A474" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B474" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="C474" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F474" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="475" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A475" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B475" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="C475" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F475" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="476" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A476" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B476" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="C476" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F476" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="477" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A477" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B477" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="C477" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F477" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="478" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A478" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B478" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="C478" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F478" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="479" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A479" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B479" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="C479" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F479" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="480" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A480" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B480" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="C480" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="F480" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="481" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A481" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B481" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C481" s="1" t="n">
+        <v>93</v>
+      </c>
+      <c r="F481" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="482" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A482" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B482" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C482" s="1" t="n">
+        <v>93</v>
+      </c>
+      <c r="F482" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="483" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A483" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B483" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C483" s="1" t="n">
+        <v>93</v>
+      </c>
+      <c r="F483" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="484" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A484" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B484" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C484" s="1" t="n">
+        <v>93</v>
+      </c>
+      <c r="F484" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="485" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A485" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B485" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C485" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="F485" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="486" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A486" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B486" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C486" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="F486" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="487" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A487" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B487" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="C487" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="F487" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="488" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A488" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B488" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="C488" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="F488" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="489" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A489" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B489" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="C489" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="F489" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="490" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A490" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B490" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="C490" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="F490" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="491" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A491" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B491" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="C491" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="F491" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="492" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A492" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B492" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="C492" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="F492" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="493" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A493" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B493" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="C493" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="F493" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="494" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A494" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B494" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="C494" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="F494" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="495" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A495" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B495" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="C495" s="1" t="n">
+        <v>91</v>
+      </c>
+      <c r="F495" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="496" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A496" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B496" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C496" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="F496" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="497" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A497" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B497" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C497" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="F497" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="498" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A498" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B498" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C498" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="F498" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="499" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A499" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B499" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C499" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="F499" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="500" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A500" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B500" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C500" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="F500" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="501" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A501" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B501" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C501" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="F501" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="502" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A502" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B502" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="C502" s="1" t="n">
+        <v>89</v>
+      </c>
+      <c r="F502" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="503" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A503" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B503" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="C503" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="F503" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="504" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A504" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B504" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="C504" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="F504" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="505" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A505" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B505" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="C505" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="F505" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="506" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A506" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B506" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="C506" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="F506" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="507" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A507" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B507" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="C507" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="F507" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="508" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A508" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B508" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="C508" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="F508" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="509" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A509" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B509" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="C509" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="F509" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="510" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A510" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B510" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="C510" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="F510" s="6" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -10069,16 +10709,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10089,7 +10729,7 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>32</v>
@@ -10100,10 +10740,10 @@
         <v>35</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>32</v>
@@ -10114,10 +10754,10 @@
         <v>36</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>32</v>
@@ -10128,10 +10768,10 @@
         <v>37</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>32</v>
@@ -10142,10 +10782,10 @@
         <v>38</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>32</v>
@@ -10159,7 +10799,7 @@
         <v>21</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>32</v>
@@ -10173,7 +10813,7 @@
         <v>15</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>32</v>
@@ -10187,7 +10827,7 @@
         <v>27</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>32</v>
@@ -10201,7 +10841,7 @@
         <v>26</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>32</v>
@@ -10212,10 +10852,10 @@
         <v>63</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>32</v>
@@ -10229,7 +10869,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>32</v>
@@ -10240,10 +10880,10 @@
         <v>67</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>32</v>
@@ -10254,10 +10894,10 @@
         <v>68</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>32</v>
@@ -10268,10 +10908,10 @@
         <v>69</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>32</v>
@@ -10282,10 +10922,10 @@
         <v>70</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>32</v>
@@ -10296,10 +10936,10 @@
         <v>71</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>32</v>
@@ -10310,10 +10950,10 @@
         <v>73</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>32</v>
@@ -10327,7 +10967,7 @@
         <v>20</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>32</v>
@@ -10341,7 +10981,7 @@
         <v>23</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>32</v>
@@ -10355,7 +10995,7 @@
         <v>24</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>32</v>
@@ -10369,7 +11009,7 @@
         <v>32</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>32</v>
@@ -10380,10 +11020,10 @@
         <v>114</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>32</v>
@@ -10397,7 +11037,7 @@
         <v>34</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>32</v>
@@ -10411,7 +11051,7 @@
         <v>45</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>32</v>
@@ -10425,7 +11065,7 @@
         <v>47</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>32</v>
@@ -10436,10 +11076,10 @@
         <v>118</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>78</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>32</v>
@@ -10453,7 +11093,7 @@
         <v>44</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>32</v>
@@ -10464,13 +11104,13 @@
         <v>127</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10478,13 +11118,13 @@
         <v>128</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10492,13 +11132,13 @@
         <v>129</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10506,13 +11146,13 @@
         <v>137</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10520,10 +11160,10 @@
         <v>155</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>32</v>
@@ -10534,13 +11174,13 @@
         <v>367</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10663,25 +11303,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>32</v>
@@ -10690,10 +11330,10 @@
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D3" s="13" t="s">
         <v>32</v>
@@ -10702,10 +11342,10 @@
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>32</v>
@@ -10717,7 +11357,7 @@
         <v>14</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>32</v>
@@ -10726,10 +11366,10 @@
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>32</v>
@@ -10738,10 +11378,10 @@
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>32</v>
@@ -10753,7 +11393,7 @@
         <v>28</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>32</v>
@@ -10762,10 +11402,10 @@
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>32</v>
@@ -10774,10 +11414,10 @@
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D10" s="13" t="s">
         <v>32</v>
@@ -10786,10 +11426,10 @@
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1"/>
       <c r="B11" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>32</v>
@@ -10798,10 +11438,10 @@
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>32</v>
@@ -10810,10 +11450,10 @@
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>32</v>
@@ -10822,10 +11462,10 @@
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>32</v>
@@ -10834,10 +11474,10 @@
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>32</v>
@@ -10846,10 +11486,10 @@
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>32</v>
@@ -10858,10 +11498,10 @@
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>32</v>
@@ -10870,10 +11510,10 @@
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>32</v>
@@ -10882,10 +11522,10 @@
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>32</v>
@@ -10894,10 +11534,10 @@
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>32</v>
@@ -10906,10 +11546,10 @@
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D21" s="13" t="s">
         <v>32</v>
@@ -10918,10 +11558,10 @@
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D22" s="13" t="s">
         <v>32</v>
@@ -10930,10 +11570,10 @@
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>32</v>
@@ -10942,10 +11582,10 @@
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D24" s="13" t="s">
         <v>32</v>
@@ -10954,10 +11594,10 @@
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D25" s="13" t="s">
         <v>32</v>
@@ -10966,10 +11606,10 @@
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1"/>
       <c r="B26" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D26" s="13" t="s">
         <v>32</v>
@@ -10978,10 +11618,10 @@
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D27" s="13" t="s">
         <v>32</v>
@@ -10990,10 +11630,10 @@
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D28" s="13" t="s">
         <v>32</v>
@@ -11002,10 +11642,10 @@
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1"/>
       <c r="B29" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D29" s="13" t="s">
         <v>32</v>
@@ -11014,10 +11654,10 @@
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D30" s="13" t="s">
         <v>32</v>
@@ -11026,10 +11666,10 @@
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D31" s="13" t="s">
         <v>32</v>
@@ -11038,10 +11678,10 @@
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1"/>
       <c r="B32" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Temmuz 2025 katsayıları işlendi.
</commit_message>
<xml_diff>
--- a/maas_verileri.xlsx
+++ b/maas_verileri.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId3"/>
@@ -657,7 +657,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="1" style="1" width="7.22"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="11" style="1" width="11.52"/>
@@ -1116,8 +1116,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D43"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="10.46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="15.14"/>
@@ -1711,6 +1711,20 @@
       </c>
       <c r="D42" s="2" t="n">
         <v>15.848415</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>1.170211</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>0.371113</v>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>18.316014</v>
       </c>
     </row>
   </sheetData>
@@ -1730,7 +1744,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G83"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="35.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="6.98"/>
@@ -2678,7 +2692,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M510"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="14.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.85"/>
@@ -10698,7 +10712,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D65"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="33.39"/>
@@ -11293,7 +11307,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D33"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="13.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="30.78"/>

</xml_diff>

<commit_message>
Bazı unvanların tazminat puanları düzeltildi.
</commit_message>
<xml_diff>
--- a/maas_verileri.xlsx
+++ b/maas_verileri.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId3"/>
@@ -2022,15 +2022,13 @@
         <v>1</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>750</v>
-      </c>
-      <c r="D16" s="7" t="n">
         <v>500</v>
       </c>
-      <c r="E16" s="7" t="n">
-        <v>750</v>
-      </c>
-      <c r="F16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7" t="n">
+        <v>375</v>
+      </c>
       <c r="G16" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2458,7 +2456,7 @@
         <v>5</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="D42" s="7"/>
       <c r="E42" s="7" t="n">
@@ -2475,7 +2473,7 @@
         <v>6</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="D43" s="7"/>
       <c r="E43" s="7" t="n">
@@ -2492,7 +2490,7 @@
         <v>7</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="D44" s="7"/>
       <c r="E44" s="7" t="n">
@@ -2509,7 +2507,7 @@
         <v>8</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="D45" s="7"/>
       <c r="E45" s="7" t="n">
@@ -2526,7 +2524,7 @@
         <v>9</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="D46" s="7"/>
       <c r="E46" s="7" t="n">

</xml_diff>

<commit_message>
Baş Müezzin için kadro sıra no eklendi, Vekil M.K ünvanı noktalama işareti değiştirildi.
</commit_message>
<xml_diff>
--- a/maas_verileri.xlsx
+++ b/maas_verileri.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="aylik_gosterge_puanlari" sheetId="1" state="visible" r:id="rId3"/>
@@ -177,7 +177,7 @@
     <t xml:space="preserve">Vekil İ-H</t>
   </si>
   <si>
-    <t xml:space="preserve">Vekil M-K</t>
+    <t xml:space="preserve">Vekil M.K</t>
   </si>
   <si>
     <t xml:space="preserve">oht_orani</t>
@@ -258,6 +258,9 @@
     <t xml:space="preserve">İmam-Hatip</t>
   </si>
   <si>
+    <t xml:space="preserve">Baş Müezzin</t>
+  </si>
+  <si>
     <t xml:space="preserve">Müezzin-Kayyım</t>
   </si>
   <si>
@@ -307,9 +310,6 @@
   </si>
   <si>
     <t xml:space="preserve">Ayniyat Saymanı</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baş Müezzin</t>
   </si>
   <si>
     <t xml:space="preserve">Cami Rehberi</t>
@@ -11526,7 +11526,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D66"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.68"/>
@@ -11776,7 +11776,7 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>77</v>
@@ -11790,13 +11790,13 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>32</v>
@@ -11804,13 +11804,13 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>32</v>
@@ -11818,10 +11818,10 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21" s="13" t="s">
         <v>69</v>
@@ -11832,13 +11832,13 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>63</v>
+        <v>24</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>69</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>32</v>
@@ -11846,10 +11846,10 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>63</v>
@@ -11860,10 +11860,10 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>63</v>
@@ -11874,13 +11874,13 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>32</v>
@@ -11888,13 +11888,13 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>32</v>
@@ -11902,13 +11902,13 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>32</v>
@@ -11916,13 +11916,13 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>32</v>
@@ -11930,90 +11930,101 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="n">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>85</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="n">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>86</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="n">
-        <v>155</v>
+        <v>137</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="n">
-        <v>367</v>
+        <v>155</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>88</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="n">
+        <v>367</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D35" s="14"/>
+      <c r="D35" s="1" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D36" s="14"/>
@@ -12104,6 +12115,9 @@
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D65" s="14"/>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D66" s="14"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -12121,7 +12135,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="13.26"/>
@@ -12147,7 +12161,7 @@
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7"/>
       <c r="B2" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>63</v>
@@ -12159,7 +12173,7 @@
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7"/>
       <c r="B3" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>63</v>
@@ -12171,7 +12185,7 @@
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>63</v>
@@ -12186,7 +12200,7 @@
         <v>14</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>32</v>
@@ -12195,7 +12209,7 @@
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7"/>
       <c r="B6" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>63</v>
@@ -12207,7 +12221,7 @@
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7"/>
       <c r="B7" s="7" t="s">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>70</v>
@@ -12219,7 +12233,7 @@
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7"/>
       <c r="B8" s="7" t="s">
-        <v>28</v>
+        <v>95</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>70</v>
@@ -12231,10 +12245,10 @@
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7"/>
       <c r="B9" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>70</v>
+        <v>97</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>32</v>
@@ -12243,10 +12257,10 @@
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7"/>
       <c r="B10" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>97</v>
+        <v>63</v>
       </c>
       <c r="D10" s="13" t="s">
         <v>32</v>
@@ -12255,7 +12269,7 @@
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7"/>
       <c r="B11" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>63</v>
@@ -12267,10 +12281,10 @@
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7"/>
       <c r="B12" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>32</v>
@@ -12279,10 +12293,10 @@
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7"/>
       <c r="B13" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>32</v>
@@ -12291,7 +12305,7 @@
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7"/>
       <c r="B14" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>63</v>
@@ -12303,7 +12317,7 @@
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7"/>
       <c r="B15" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>63</v>
@@ -12315,7 +12329,7 @@
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7"/>
       <c r="B16" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>63</v>
@@ -12327,10 +12341,10 @@
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7"/>
       <c r="B17" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>32</v>
@@ -12339,10 +12353,10 @@
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7"/>
       <c r="B18" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>32</v>
@@ -12351,10 +12365,10 @@
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7"/>
       <c r="B19" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>32</v>
@@ -12363,7 +12377,7 @@
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7"/>
       <c r="B20" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>63</v>
@@ -12375,7 +12389,7 @@
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7"/>
       <c r="B21" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>63</v>
@@ -12387,10 +12401,10 @@
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7"/>
       <c r="B22" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D22" s="13" t="s">
         <v>32</v>
@@ -12399,10 +12413,10 @@
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7"/>
       <c r="B23" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>32</v>
@@ -12411,10 +12425,10 @@
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7"/>
       <c r="B24" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>97</v>
+        <v>63</v>
       </c>
       <c r="D24" s="13" t="s">
         <v>32</v>
@@ -12423,7 +12437,7 @@
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7"/>
       <c r="B25" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>63</v>
@@ -12435,10 +12449,10 @@
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7"/>
       <c r="B26" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D26" s="13" t="s">
         <v>32</v>
@@ -12447,7 +12461,7 @@
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7"/>
       <c r="B27" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>69</v>
@@ -12459,7 +12473,7 @@
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7"/>
       <c r="B28" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>69</v>
@@ -12471,7 +12485,7 @@
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7"/>
       <c r="B29" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>69</v>
@@ -12483,10 +12497,10 @@
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7"/>
       <c r="B30" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D30" s="13" t="s">
         <v>32</v>
@@ -12495,7 +12509,7 @@
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7"/>
       <c r="B31" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>63</v>
@@ -12506,21 +12520,9 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7"/>
-      <c r="B32" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>